<commit_message>
Commit local changes before merging chandru branch
</commit_message>
<xml_diff>
--- a/public/templates/employee_bulk_upload_template.xlsx
+++ b/public/templates/employee_bulk_upload_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="107">
   <si>
     <t>Bulk Upload Template Instructions</t>
   </si>
@@ -65,6 +65,9 @@
     <t>phone_number</t>
   </si>
   <si>
+    <t>emergency_contact_phone</t>
+  </si>
+  <si>
     <t>date_of_birth</t>
   </si>
   <si>
@@ -77,6 +80,12 @@
     <t>gender</t>
   </si>
   <si>
+    <t>blood_group</t>
+  </si>
+  <si>
+    <t>marital_status</t>
+  </si>
+  <si>
     <t>employment_model</t>
   </si>
   <si>
@@ -92,6 +101,12 @@
     <t>bank_ifsc</t>
   </si>
   <si>
+    <t>bank_name</t>
+  </si>
+  <si>
+    <t>bank_branch</t>
+  </si>
+  <si>
     <t>account_holder_name</t>
   </si>
   <si>
@@ -101,9 +116,27 @@
     <t>aadhaar_number</t>
   </si>
   <si>
+    <t>pf_applicable</t>
+  </si>
+  <si>
+    <t>uan_mode</t>
+  </si>
+  <si>
+    <t>uan_number</t>
+  </si>
+  <si>
+    <t>esi_applicable</t>
+  </si>
+  <si>
     <t>esic_number</t>
   </si>
   <si>
+    <t>pt_applicable</t>
+  </si>
+  <si>
+    <t>lwf_applicable</t>
+  </si>
+  <si>
     <t>tds_regime</t>
   </si>
   <si>
@@ -134,70 +167,172 @@
     <t>other_additions</t>
   </si>
   <si>
-    <t>pf_applicable</t>
-  </si>
-  <si>
-    <t>esi_applicable</t>
-  </si>
-  <si>
-    <t>pt_applicable</t>
-  </si>
-  <si>
-    <t>EMP-001</t>
-  </si>
-  <si>
-    <t>SYNSTAR</t>
-  </si>
-  <si>
-    <t>MB-01</t>
-  </si>
-  <si>
-    <t>John Doe</t>
-  </si>
-  <si>
-    <t>john@example.com</t>
-  </si>
-  <si>
-    <t>9876543210</t>
-  </si>
-  <si>
-    <t>1990-01-01</t>
-  </si>
-  <si>
-    <t>2023-01-01</t>
-  </si>
-  <si>
-    <t>Developer</t>
+    <t>EMP-103</t>
+  </si>
+  <si>
+    <t>SYN-STAFF-01</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Amit Patel</t>
+  </si>
+  <si>
+    <t>amit.patel103@example.com</t>
+  </si>
+  <si>
+    <t>7777123450</t>
+  </si>
+  <si>
+    <t>7777123451</t>
+  </si>
+  <si>
+    <t>1995-12-01</t>
+  </si>
+  <si>
+    <t>2023-06-01</t>
+  </si>
+  <si>
+    <t>Frontend Developer</t>
   </si>
   <si>
     <t>male</t>
   </si>
   <si>
+    <t>B+</t>
+  </si>
+  <si>
+    <t>single</t>
+  </si>
+  <si>
     <t>agency_contract</t>
   </si>
   <si>
-    <t>123 Main St</t>
-  </si>
-  <si>
-    <t>1234567890</t>
-  </si>
-  <si>
-    <t>HDFC0000001</t>
-  </si>
-  <si>
-    <t>ABCDE1234F</t>
-  </si>
-  <si>
-    <t>123412341234</t>
-  </si>
-  <si>
-    <t>1111111111</t>
+    <t>0</t>
+  </si>
+  <si>
+    <t>789 Link Road, Ahmedabad</t>
+  </si>
+  <si>
+    <t>556677889900</t>
+  </si>
+  <si>
+    <t>ICIC0005566</t>
+  </si>
+  <si>
+    <t>ICICI Bank</t>
+  </si>
+  <si>
+    <t>Ahmedabad Branch</t>
+  </si>
+  <si>
+    <t>KLMNO9012P</t>
+  </si>
+  <si>
+    <t>444455556666</t>
+  </si>
+  <si>
+    <t>1</t>
   </si>
   <si>
     <t>new</t>
   </si>
   <si>
+    <t>old</t>
+  </si>
+  <si>
     <t>part_of_ctc</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>25000</t>
+  </si>
+  <si>
+    <t>12500</t>
+  </si>
+  <si>
+    <t>1600</t>
+  </si>
+  <si>
+    <t>1250</t>
+  </si>
+  <si>
+    <t>6000</t>
+  </si>
+  <si>
+    <t>EMP-104</t>
+  </si>
+  <si>
+    <t>Sneha Desai</t>
+  </si>
+  <si>
+    <t>sneha.desai104@example.com</t>
+  </si>
+  <si>
+    <t>6666987654</t>
+  </si>
+  <si>
+    <t>6666987655</t>
+  </si>
+  <si>
+    <t>1991-03-10</t>
+  </si>
+  <si>
+    <t>2023-11-20</t>
+  </si>
+  <si>
+    <t>Product Manager</t>
+  </si>
+  <si>
+    <t>female</t>
+  </si>
+  <si>
+    <t>AB+</t>
+  </si>
+  <si>
+    <t>married</t>
+  </si>
+  <si>
+    <t>eor</t>
+  </si>
+  <si>
+    <t>321 IT Park, Bengaluru</t>
+  </si>
+  <si>
+    <t>334455667788</t>
+  </si>
+  <si>
+    <t>AXIS0003344</t>
+  </si>
+  <si>
+    <t>Axis Bank</t>
+  </si>
+  <si>
+    <t>Bengaluru Branch</t>
+  </si>
+  <si>
+    <t>QRSTU3456V</t>
+  </si>
+  <si>
+    <t>111122223333</t>
+  </si>
+  <si>
+    <t>over_and_above</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>40000</t>
+  </si>
+  <si>
+    <t>20000</t>
+  </si>
+  <si>
+    <t>8000</t>
   </si>
 </sst>
 </file>
@@ -668,19 +803,19 @@
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AF2"/>
+  <dimension ref="A1:AN3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="32" width="20" customWidth="1"/>
+    <col min="1" max="40" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>11</v>
       </c>
@@ -777,107 +912,277 @@
       <c r="AF1" s="4" t="s">
         <v>42</v>
       </c>
+      <c r="AG1" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="AH1" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="AI1" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="AJ1" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="AK1" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL1" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="AM1" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="AN1" s="4" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="J2" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="T2" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="U2" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="V2" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="W2" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="X2" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="Y2" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="Z2" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA2" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="AB2" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC2" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="AD2" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="AE2" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="AF2" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>78</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>79</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>80</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>81</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>82</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" t="s">
         <v>52</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="C3" t="s">
         <v>53</v>
       </c>
-      <c r="L2" s="5">
-        <v>0</v>
-      </c>
-      <c r="M2" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="N2" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="O2" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="P2" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q2" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="R2" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="S2" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="T2" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="U2" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="V2" s="5">
-        <v>26</v>
-      </c>
-      <c r="W2" s="5">
-        <v>15000</v>
-      </c>
-      <c r="X2" s="5">
-        <v>5000</v>
-      </c>
-      <c r="Y2" s="5">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="5">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="5">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="5">
-        <v>0</v>
-      </c>
-      <c r="AD2" s="5">
-        <v>1</v>
-      </c>
-      <c r="AE2" s="5">
-        <v>1</v>
-      </c>
-      <c r="AF2" s="5">
-        <v>1</v>
+      <c r="D3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F3" t="s">
+        <v>86</v>
+      </c>
+      <c r="G3" t="s">
+        <v>87</v>
+      </c>
+      <c r="H3" t="s">
+        <v>88</v>
+      </c>
+      <c r="I3" t="s">
+        <v>89</v>
+      </c>
+      <c r="J3" t="s">
+        <v>90</v>
+      </c>
+      <c r="K3" t="s">
+        <v>91</v>
+      </c>
+      <c r="L3" t="s">
+        <v>92</v>
+      </c>
+      <c r="M3" t="s">
+        <v>93</v>
+      </c>
+      <c r="N3" t="s">
+        <v>94</v>
+      </c>
+      <c r="O3" t="s">
+        <v>73</v>
+      </c>
+      <c r="P3" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>96</v>
+      </c>
+      <c r="R3" t="s">
+        <v>97</v>
+      </c>
+      <c r="S3" t="s">
+        <v>98</v>
+      </c>
+      <c r="T3" t="s">
+        <v>99</v>
+      </c>
+      <c r="U3" t="s">
+        <v>84</v>
+      </c>
+      <c r="V3" t="s">
+        <v>100</v>
+      </c>
+      <c r="W3" t="s">
+        <v>101</v>
+      </c>
+      <c r="X3" t="s">
+        <v>73</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>74</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>73</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>73</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>74</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>102</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>103</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>104</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>105</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>80</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>81</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>106</v>
+      </c>
+      <c r="AN3" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Merge rajesh employee portal with chandru auth/settings work
</commit_message>
<xml_diff>
--- a/public/templates/employee_bulk_upload_template.xlsx
+++ b/public/templates/employee_bulk_upload_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="107">
   <si>
     <t>Bulk Upload Template Instructions</t>
   </si>
@@ -65,6 +65,9 @@
     <t>phone_number</t>
   </si>
   <si>
+    <t>emergency_contact_phone</t>
+  </si>
+  <si>
     <t>date_of_birth</t>
   </si>
   <si>
@@ -77,6 +80,12 @@
     <t>gender</t>
   </si>
   <si>
+    <t>blood_group</t>
+  </si>
+  <si>
+    <t>marital_status</t>
+  </si>
+  <si>
     <t>employment_model</t>
   </si>
   <si>
@@ -92,6 +101,12 @@
     <t>bank_ifsc</t>
   </si>
   <si>
+    <t>bank_name</t>
+  </si>
+  <si>
+    <t>bank_branch</t>
+  </si>
+  <si>
     <t>account_holder_name</t>
   </si>
   <si>
@@ -101,9 +116,27 @@
     <t>aadhaar_number</t>
   </si>
   <si>
+    <t>pf_applicable</t>
+  </si>
+  <si>
+    <t>uan_mode</t>
+  </si>
+  <si>
+    <t>uan_number</t>
+  </si>
+  <si>
+    <t>esi_applicable</t>
+  </si>
+  <si>
     <t>esic_number</t>
   </si>
   <si>
+    <t>pt_applicable</t>
+  </si>
+  <si>
+    <t>lwf_applicable</t>
+  </si>
+  <si>
     <t>tds_regime</t>
   </si>
   <si>
@@ -134,70 +167,172 @@
     <t>other_additions</t>
   </si>
   <si>
-    <t>pf_applicable</t>
-  </si>
-  <si>
-    <t>esi_applicable</t>
-  </si>
-  <si>
-    <t>pt_applicable</t>
-  </si>
-  <si>
-    <t>EMP-001</t>
-  </si>
-  <si>
-    <t>SYNSTAR</t>
-  </si>
-  <si>
-    <t>MB-01</t>
-  </si>
-  <si>
-    <t>John Doe</t>
-  </si>
-  <si>
-    <t>john@example.com</t>
-  </si>
-  <si>
-    <t>9876543210</t>
-  </si>
-  <si>
-    <t>1990-01-01</t>
-  </si>
-  <si>
-    <t>2023-01-01</t>
-  </si>
-  <si>
-    <t>Developer</t>
+    <t>EMP-103</t>
+  </si>
+  <si>
+    <t>SYN-STAFF-01</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Amit Patel</t>
+  </si>
+  <si>
+    <t>amit.patel103@example.com</t>
+  </si>
+  <si>
+    <t>7777123450</t>
+  </si>
+  <si>
+    <t>7777123451</t>
+  </si>
+  <si>
+    <t>1995-12-01</t>
+  </si>
+  <si>
+    <t>2023-06-01</t>
+  </si>
+  <si>
+    <t>Frontend Developer</t>
   </si>
   <si>
     <t>male</t>
   </si>
   <si>
+    <t>B+</t>
+  </si>
+  <si>
+    <t>single</t>
+  </si>
+  <si>
     <t>agency_contract</t>
   </si>
   <si>
-    <t>123 Main St</t>
-  </si>
-  <si>
-    <t>1234567890</t>
-  </si>
-  <si>
-    <t>HDFC0000001</t>
-  </si>
-  <si>
-    <t>ABCDE1234F</t>
-  </si>
-  <si>
-    <t>123412341234</t>
-  </si>
-  <si>
-    <t>1111111111</t>
+    <t>0</t>
+  </si>
+  <si>
+    <t>789 Link Road, Ahmedabad</t>
+  </si>
+  <si>
+    <t>556677889900</t>
+  </si>
+  <si>
+    <t>ICIC0005566</t>
+  </si>
+  <si>
+    <t>ICICI Bank</t>
+  </si>
+  <si>
+    <t>Ahmedabad Branch</t>
+  </si>
+  <si>
+    <t>KLMNO9012P</t>
+  </si>
+  <si>
+    <t>444455556666</t>
+  </si>
+  <si>
+    <t>1</t>
   </si>
   <si>
     <t>new</t>
   </si>
   <si>
+    <t>old</t>
+  </si>
+  <si>
     <t>part_of_ctc</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>25000</t>
+  </si>
+  <si>
+    <t>12500</t>
+  </si>
+  <si>
+    <t>1600</t>
+  </si>
+  <si>
+    <t>1250</t>
+  </si>
+  <si>
+    <t>6000</t>
+  </si>
+  <si>
+    <t>EMP-104</t>
+  </si>
+  <si>
+    <t>Sneha Desai</t>
+  </si>
+  <si>
+    <t>sneha.desai104@example.com</t>
+  </si>
+  <si>
+    <t>6666987654</t>
+  </si>
+  <si>
+    <t>6666987655</t>
+  </si>
+  <si>
+    <t>1991-03-10</t>
+  </si>
+  <si>
+    <t>2023-11-20</t>
+  </si>
+  <si>
+    <t>Product Manager</t>
+  </si>
+  <si>
+    <t>female</t>
+  </si>
+  <si>
+    <t>AB+</t>
+  </si>
+  <si>
+    <t>married</t>
+  </si>
+  <si>
+    <t>eor</t>
+  </si>
+  <si>
+    <t>321 IT Park, Bengaluru</t>
+  </si>
+  <si>
+    <t>334455667788</t>
+  </si>
+  <si>
+    <t>AXIS0003344</t>
+  </si>
+  <si>
+    <t>Axis Bank</t>
+  </si>
+  <si>
+    <t>Bengaluru Branch</t>
+  </si>
+  <si>
+    <t>QRSTU3456V</t>
+  </si>
+  <si>
+    <t>111122223333</t>
+  </si>
+  <si>
+    <t>over_and_above</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>40000</t>
+  </si>
+  <si>
+    <t>20000</t>
+  </si>
+  <si>
+    <t>8000</t>
   </si>
 </sst>
 </file>
@@ -668,19 +803,19 @@
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AF2"/>
+  <dimension ref="A1:AN3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="32" width="20" customWidth="1"/>
+    <col min="1" max="40" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>11</v>
       </c>
@@ -777,107 +912,277 @@
       <c r="AF1" s="4" t="s">
         <v>42</v>
       </c>
+      <c r="AG1" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="AH1" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="AI1" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="AJ1" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="AK1" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL1" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="AM1" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="AN1" s="4" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="J2" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="T2" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="U2" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="V2" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="W2" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="X2" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="Y2" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="Z2" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA2" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="AB2" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC2" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="AD2" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="AE2" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="AF2" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>78</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>79</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>80</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>81</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>82</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" t="s">
         <v>52</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="C3" t="s">
         <v>53</v>
       </c>
-      <c r="L2" s="5">
-        <v>0</v>
-      </c>
-      <c r="M2" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="N2" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="O2" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="P2" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q2" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="R2" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="S2" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="T2" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="U2" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="V2" s="5">
-        <v>26</v>
-      </c>
-      <c r="W2" s="5">
-        <v>15000</v>
-      </c>
-      <c r="X2" s="5">
-        <v>5000</v>
-      </c>
-      <c r="Y2" s="5">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="5">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="5">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="5">
-        <v>0</v>
-      </c>
-      <c r="AD2" s="5">
-        <v>1</v>
-      </c>
-      <c r="AE2" s="5">
-        <v>1</v>
-      </c>
-      <c r="AF2" s="5">
-        <v>1</v>
+      <c r="D3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F3" t="s">
+        <v>86</v>
+      </c>
+      <c r="G3" t="s">
+        <v>87</v>
+      </c>
+      <c r="H3" t="s">
+        <v>88</v>
+      </c>
+      <c r="I3" t="s">
+        <v>89</v>
+      </c>
+      <c r="J3" t="s">
+        <v>90</v>
+      </c>
+      <c r="K3" t="s">
+        <v>91</v>
+      </c>
+      <c r="L3" t="s">
+        <v>92</v>
+      </c>
+      <c r="M3" t="s">
+        <v>93</v>
+      </c>
+      <c r="N3" t="s">
+        <v>94</v>
+      </c>
+      <c r="O3" t="s">
+        <v>73</v>
+      </c>
+      <c r="P3" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>96</v>
+      </c>
+      <c r="R3" t="s">
+        <v>97</v>
+      </c>
+      <c r="S3" t="s">
+        <v>98</v>
+      </c>
+      <c r="T3" t="s">
+        <v>99</v>
+      </c>
+      <c r="U3" t="s">
+        <v>84</v>
+      </c>
+      <c r="V3" t="s">
+        <v>100</v>
+      </c>
+      <c r="W3" t="s">
+        <v>101</v>
+      </c>
+      <c r="X3" t="s">
+        <v>73</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>74</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>73</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>73</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>74</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>102</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>103</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>104</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>105</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>80</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>81</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>106</v>
+      </c>
+      <c r="AN3" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: resolve employee form validation issues, add live checkUnique endpoint, fix bank change request approvals and client onboarding redirect
</commit_message>
<xml_diff>
--- a/public/templates/employee_bulk_upload_template.xlsx
+++ b/public/templates/employee_bulk_upload_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="72">
   <si>
     <t>Bulk Upload Template Instructions</t>
   </si>
@@ -65,7 +65,7 @@
     <t>phone_number</t>
   </si>
   <si>
-    <t>emergency_contact_phone</t>
+    <t>emergency_contact_name</t>
   </si>
   <si>
     <t>date_of_birth</t>
@@ -74,24 +74,30 @@
     <t>date_of_joining</t>
   </si>
   <si>
+    <t>probation_end_date</t>
+  </si>
+  <si>
     <t>designation</t>
   </si>
   <si>
     <t>gender</t>
   </si>
   <si>
-    <t>blood_group</t>
-  </si>
-  <si>
-    <t>marital_status</t>
-  </si>
-  <si>
     <t>employment_model</t>
   </si>
   <si>
     <t>prior_employment_flag</t>
   </si>
   <si>
+    <t>previous_employer_name</t>
+  </si>
+  <si>
+    <t>previous_employer_uan</t>
+  </si>
+  <si>
+    <t>reporting_manager_code</t>
+  </si>
+  <si>
     <t>residential_address</t>
   </si>
   <si>
@@ -101,12 +107,6 @@
     <t>bank_ifsc</t>
   </si>
   <si>
-    <t>bank_name</t>
-  </si>
-  <si>
-    <t>bank_branch</t>
-  </si>
-  <si>
     <t>account_holder_name</t>
   </si>
   <si>
@@ -116,223 +116,118 @@
     <t>aadhaar_number</t>
   </si>
   <si>
+    <t>esic_number</t>
+  </si>
+  <si>
+    <t>esi_contribution_period_end</t>
+  </si>
+  <si>
+    <t>declarations_accepted</t>
+  </si>
+  <si>
+    <t>tds_regime</t>
+  </si>
+  <si>
+    <t>gratuity_mode</t>
+  </si>
+  <si>
+    <t>lop_basis_days</t>
+  </si>
+  <si>
+    <t>basic_pay</t>
+  </si>
+  <si>
+    <t>hra</t>
+  </si>
+  <si>
+    <t>conveyance</t>
+  </si>
+  <si>
+    <t>da</t>
+  </si>
+  <si>
+    <t>medical_allowance</t>
+  </si>
+  <si>
+    <t>special_allowance</t>
+  </si>
+  <si>
+    <t>other_additions</t>
+  </si>
+  <si>
     <t>pf_applicable</t>
   </si>
   <si>
-    <t>uan_mode</t>
-  </si>
-  <si>
-    <t>uan_number</t>
-  </si>
-  <si>
     <t>esi_applicable</t>
   </si>
   <si>
-    <t>esic_number</t>
-  </si>
-  <si>
     <t>pt_applicable</t>
   </si>
   <si>
-    <t>lwf_applicable</t>
-  </si>
-  <si>
-    <t>tds_regime</t>
-  </si>
-  <si>
-    <t>gratuity_mode</t>
-  </si>
-  <si>
-    <t>lop_basis_days</t>
-  </si>
-  <si>
-    <t>basic_pay</t>
-  </si>
-  <si>
-    <t>hra</t>
-  </si>
-  <si>
-    <t>conveyance</t>
-  </si>
-  <si>
-    <t>da</t>
-  </si>
-  <si>
-    <t>medical_allowance</t>
-  </si>
-  <si>
-    <t>special_allowance</t>
-  </si>
-  <si>
-    <t>other_additions</t>
-  </si>
-  <si>
-    <t>EMP-103</t>
-  </si>
-  <si>
-    <t>SYN-STAFF-01</t>
+    <t>EMP-001</t>
+  </si>
+  <si>
+    <t>SYNSTAR</t>
+  </si>
+  <si>
+    <t>MB-01</t>
+  </si>
+  <si>
+    <t>John Doe</t>
+  </si>
+  <si>
+    <t>john@example.com</t>
+  </si>
+  <si>
+    <t>9876543210</t>
+  </si>
+  <si>
+    <t>Robert Smith</t>
+  </si>
+  <si>
+    <t>1990-01-01</t>
+  </si>
+  <si>
+    <t>2023-01-01</t>
+  </si>
+  <si>
+    <t>2023-06-30</t>
+  </si>
+  <si>
+    <t>Developer</t>
+  </si>
+  <si>
+    <t>male</t>
+  </si>
+  <si>
+    <t>agency_contract</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>Amit Patel</t>
-  </si>
-  <si>
-    <t>amit.patel103@example.com</t>
-  </si>
-  <si>
-    <t>7777123450</t>
-  </si>
-  <si>
-    <t>7777123451</t>
-  </si>
-  <si>
-    <t>1995-12-01</t>
-  </si>
-  <si>
-    <t>2023-06-01</t>
-  </si>
-  <si>
-    <t>Frontend Developer</t>
-  </si>
-  <si>
-    <t>male</t>
-  </si>
-  <si>
-    <t>B+</t>
-  </si>
-  <si>
-    <t>single</t>
-  </si>
-  <si>
-    <t>agency_contract</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>789 Link Road, Ahmedabad</t>
-  </si>
-  <si>
-    <t>556677889900</t>
-  </si>
-  <si>
-    <t>ICIC0005566</t>
-  </si>
-  <si>
-    <t>ICICI Bank</t>
-  </si>
-  <si>
-    <t>Ahmedabad Branch</t>
-  </si>
-  <si>
-    <t>KLMNO9012P</t>
-  </si>
-  <si>
-    <t>444455556666</t>
-  </si>
-  <si>
-    <t>1</t>
+    <t>123 Main St</t>
+  </si>
+  <si>
+    <t>1234567890</t>
+  </si>
+  <si>
+    <t>HDFC0000001</t>
+  </si>
+  <si>
+    <t>ABCDE1234F</t>
+  </si>
+  <si>
+    <t>123412341234</t>
+  </si>
+  <si>
+    <t>1111111111</t>
   </si>
   <si>
     <t>new</t>
   </si>
   <si>
-    <t>old</t>
-  </si>
-  <si>
     <t>part_of_ctc</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>25000</t>
-  </si>
-  <si>
-    <t>12500</t>
-  </si>
-  <si>
-    <t>1600</t>
-  </si>
-  <si>
-    <t>1250</t>
-  </si>
-  <si>
-    <t>6000</t>
-  </si>
-  <si>
-    <t>EMP-104</t>
-  </si>
-  <si>
-    <t>Sneha Desai</t>
-  </si>
-  <si>
-    <t>sneha.desai104@example.com</t>
-  </si>
-  <si>
-    <t>6666987654</t>
-  </si>
-  <si>
-    <t>6666987655</t>
-  </si>
-  <si>
-    <t>1991-03-10</t>
-  </si>
-  <si>
-    <t>2023-11-20</t>
-  </si>
-  <si>
-    <t>Product Manager</t>
-  </si>
-  <si>
-    <t>female</t>
-  </si>
-  <si>
-    <t>AB+</t>
-  </si>
-  <si>
-    <t>married</t>
-  </si>
-  <si>
-    <t>eor</t>
-  </si>
-  <si>
-    <t>321 IT Park, Bengaluru</t>
-  </si>
-  <si>
-    <t>334455667788</t>
-  </si>
-  <si>
-    <t>AXIS0003344</t>
-  </si>
-  <si>
-    <t>Axis Bank</t>
-  </si>
-  <si>
-    <t>Bengaluru Branch</t>
-  </si>
-  <si>
-    <t>QRSTU3456V</t>
-  </si>
-  <si>
-    <t>111122223333</t>
-  </si>
-  <si>
-    <t>over_and_above</t>
-  </si>
-  <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>40000</t>
-  </si>
-  <si>
-    <t>20000</t>
-  </si>
-  <si>
-    <t>8000</t>
   </si>
 </sst>
 </file>
@@ -803,19 +698,19 @@
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AN3"/>
+  <dimension ref="A1:AM2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="40" width="20" customWidth="1"/>
+    <col min="1" max="39" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>11</v>
       </c>
@@ -933,256 +828,128 @@
       <c r="AM1" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="AN1" s="4" t="s">
+    </row>
+    <row r="2" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="2" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="B2" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="G2" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="H2" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="I2" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="J2" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="K2" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="L2" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="M2" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="N2" s="5">
+        <v>0</v>
+      </c>
+      <c r="O2" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="P2" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="R2" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="S2" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="T2" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="Q2" s="5" t="s">
+      <c r="U2" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="V2" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="R2" s="5" t="s">
+      <c r="W2" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="S2" s="5" t="s">
+      <c r="X2" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="T2" s="5" t="s">
+      <c r="Y2" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="Z2" s="5">
+        <v>1</v>
+      </c>
+      <c r="AA2" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="U2" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="V2" s="5" t="s">
+      <c r="AB2" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="W2" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="X2" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="Y2" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="Z2" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="AA2" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="AB2" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC2" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="AD2" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="AE2" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="AF2" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>77</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>78</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>79</v>
-      </c>
-      <c r="AJ2" t="s">
-        <v>80</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>65</v>
-      </c>
-      <c r="AL2" t="s">
-        <v>81</v>
-      </c>
-      <c r="AM2" t="s">
-        <v>82</v>
-      </c>
-      <c r="AN2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="3" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>83</v>
-      </c>
-      <c r="B3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C3" t="s">
-        <v>53</v>
-      </c>
-      <c r="D3" t="s">
-        <v>84</v>
-      </c>
-      <c r="E3" t="s">
-        <v>85</v>
-      </c>
-      <c r="F3" t="s">
-        <v>86</v>
-      </c>
-      <c r="G3" t="s">
-        <v>87</v>
-      </c>
-      <c r="H3" t="s">
-        <v>88</v>
-      </c>
-      <c r="I3" t="s">
-        <v>89</v>
-      </c>
-      <c r="J3" t="s">
-        <v>90</v>
-      </c>
-      <c r="K3" t="s">
-        <v>91</v>
-      </c>
-      <c r="L3" t="s">
-        <v>92</v>
-      </c>
-      <c r="M3" t="s">
-        <v>93</v>
-      </c>
-      <c r="N3" t="s">
-        <v>94</v>
-      </c>
-      <c r="O3" t="s">
-        <v>73</v>
-      </c>
-      <c r="P3" t="s">
-        <v>95</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>96</v>
-      </c>
-      <c r="R3" t="s">
-        <v>97</v>
-      </c>
-      <c r="S3" t="s">
-        <v>98</v>
-      </c>
-      <c r="T3" t="s">
-        <v>99</v>
-      </c>
-      <c r="U3" t="s">
-        <v>84</v>
-      </c>
-      <c r="V3" t="s">
-        <v>100</v>
-      </c>
-      <c r="W3" t="s">
-        <v>101</v>
-      </c>
-      <c r="X3" t="s">
-        <v>73</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>74</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>65</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>73</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>73</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>74</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>102</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>103</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>104</v>
-      </c>
-      <c r="AI3" t="s">
-        <v>105</v>
-      </c>
-      <c r="AJ3" t="s">
-        <v>80</v>
-      </c>
-      <c r="AK3" t="s">
-        <v>65</v>
-      </c>
-      <c r="AL3" t="s">
-        <v>81</v>
-      </c>
-      <c r="AM3" t="s">
-        <v>106</v>
-      </c>
-      <c r="AN3" t="s">
-        <v>65</v>
+      <c r="AC2" s="5">
+        <v>26</v>
+      </c>
+      <c r="AD2" s="5">
+        <v>15000</v>
+      </c>
+      <c r="AE2" s="5">
+        <v>5000</v>
+      </c>
+      <c r="AF2" s="5">
+        <v>0</v>
+      </c>
+      <c r="AG2" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH2" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI2" s="5">
+        <v>0</v>
+      </c>
+      <c r="AJ2" s="5">
+        <v>0</v>
+      </c>
+      <c r="AK2" s="5">
+        <v>1</v>
+      </c>
+      <c r="AL2" s="5">
+        <v>1</v>
+      </c>
+      <c r="AM2" s="5">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>